<commit_message>
lots of new data
</commit_message>
<xml_diff>
--- a/data/community_fall2026.xlsx
+++ b/data/community_fall2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernbromley/Desktop/AVCA_BANWR/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8DC3FCA-3652-444C-988F-D99DAC342A82}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{792B1686-1F6D-C343-ADC4-DAB68D1987DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" xr2:uid="{7D6DEC84-1D80-5044-AEB0-AE046E367DDB}"/>
   </bookViews>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="81">
   <si>
     <t>plot</t>
   </si>
@@ -228,6 +228,114 @@
   </si>
   <si>
     <t>DESCOO</t>
+  </si>
+  <si>
+    <t>C23</t>
+  </si>
+  <si>
+    <t>ERIOGspp</t>
+  </si>
+  <si>
+    <t>ENNDES</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>CARARI</t>
+  </si>
+  <si>
+    <t>C36</t>
+  </si>
+  <si>
+    <t>ERACUR</t>
+  </si>
+  <si>
+    <t>C26</t>
+  </si>
+  <si>
+    <t>RHYPHY</t>
+  </si>
+  <si>
+    <t>AMAPAL</t>
+  </si>
+  <si>
+    <t>VICLUD</t>
+  </si>
+  <si>
+    <t>C48</t>
+  </si>
+  <si>
+    <t>ALLINC</t>
+  </si>
+  <si>
+    <t>C24</t>
+  </si>
+  <si>
+    <t>C22</t>
+  </si>
+  <si>
+    <t>C18</t>
+  </si>
+  <si>
+    <t>C34</t>
+  </si>
+  <si>
+    <t>C33</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C4</t>
+  </si>
+  <si>
+    <t>C49</t>
+  </si>
+  <si>
+    <t>C40</t>
+  </si>
+  <si>
+    <t>C27</t>
+  </si>
+  <si>
+    <t>C14</t>
+  </si>
+  <si>
+    <t>C28</t>
+  </si>
+  <si>
+    <t>C21</t>
+  </si>
+  <si>
+    <t>EVOARI</t>
+  </si>
+  <si>
+    <t>C43</t>
+  </si>
+  <si>
+    <t>C7</t>
+  </si>
+  <si>
+    <t>C16</t>
+  </si>
+  <si>
+    <t>C50</t>
+  </si>
+  <si>
+    <t>C44</t>
+  </si>
+  <si>
+    <t>ALLIUspp</t>
+  </si>
+  <si>
+    <t>C25</t>
+  </si>
+  <si>
+    <t>BOUREP</t>
+  </si>
+  <si>
+    <t>C32</t>
   </si>
 </sst>
 </file>
@@ -632,10 +740,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD559584-3F3E-3149-A2F9-E170630AB5BF}">
-  <dimension ref="A1:AT50"/>
+  <dimension ref="A1:BE75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -774,8 +882,41 @@
       <c r="AT1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:46" x14ac:dyDescent="0.2">
+      <c r="AU1" t="s">
+        <v>46</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>47</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>54</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>55</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>57</v>
+      </c>
+      <c r="BC1" t="s">
+        <v>71</v>
+      </c>
+      <c r="BD1" t="s">
+        <v>77</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>97</v>
       </c>
@@ -844,7 +985,7 @@
       <c r="AJ2" s="1"/>
       <c r="AK2" s="1"/>
     </row>
-    <row r="3" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>65</v>
       </c>
@@ -913,7 +1054,7 @@
       <c r="AJ3" s="1"/>
       <c r="AK3" s="1"/>
     </row>
-    <row r="4" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>68</v>
       </c>
@@ -982,7 +1123,7 @@
       <c r="AJ4" s="1"/>
       <c r="AK4" s="1"/>
     </row>
-    <row r="5" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>74</v>
       </c>
@@ -1051,7 +1192,7 @@
       <c r="AJ5" s="1"/>
       <c r="AK5" s="1"/>
     </row>
-    <row r="6" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>55</v>
       </c>
@@ -1106,7 +1247,7 @@
       <c r="AJ6" s="1"/>
       <c r="AK6" s="1"/>
     </row>
-    <row r="7" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>61</v>
       </c>
@@ -1163,7 +1304,7 @@
       <c r="AJ7" s="1"/>
       <c r="AK7" s="1"/>
     </row>
-    <row r="8" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>57</v>
       </c>
@@ -1222,7 +1363,7 @@
       <c r="AJ8" s="1"/>
       <c r="AK8" s="1"/>
     </row>
-    <row r="9" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>84</v>
       </c>
@@ -1271,7 +1412,7 @@
       <c r="AJ9" s="1"/>
       <c r="AK9" s="1"/>
     </row>
-    <row r="10" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>94</v>
       </c>
@@ -1324,7 +1465,7 @@
       <c r="AJ10" s="1"/>
       <c r="AK10" s="1"/>
     </row>
-    <row r="11" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>67</v>
       </c>
@@ -1373,7 +1514,7 @@
       <c r="AJ11" s="1"/>
       <c r="AK11" s="1"/>
     </row>
-    <row r="12" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>88</v>
       </c>
@@ -1420,7 +1561,7 @@
       <c r="AJ12" s="1"/>
       <c r="AK12" s="1"/>
     </row>
-    <row r="13" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>91</v>
       </c>
@@ -1475,7 +1616,7 @@
       <c r="AJ13" s="1"/>
       <c r="AK13" s="1"/>
     </row>
-    <row r="14" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>63</v>
       </c>
@@ -1528,7 +1669,7 @@
       <c r="AJ14" s="1"/>
       <c r="AK14" s="1"/>
     </row>
-    <row r="15" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>89</v>
       </c>
@@ -1577,7 +1718,7 @@
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
     </row>
-    <row r="16" spans="1:46" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:57" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>49</v>
       </c>
@@ -1626,7 +1767,7 @@
       <c r="AJ16" s="1"/>
       <c r="AK16" s="1"/>
     </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>72</v>
       </c>
@@ -1673,7 +1814,7 @@
       <c r="AJ17" s="1"/>
       <c r="AK17" s="1"/>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>14</v>
       </c>
@@ -1716,7 +1857,7 @@
       <c r="AJ18" s="1"/>
       <c r="AK18" s="1"/>
     </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>40</v>
       </c>
@@ -1765,7 +1906,7 @@
       <c r="AJ19" s="1"/>
       <c r="AK19" s="1"/>
     </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>22</v>
       </c>
@@ -1828,7 +1969,7 @@
       <c r="AJ20" s="1"/>
       <c r="AK20" s="1"/>
     </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>21</v>
       </c>
@@ -1885,7 +2026,7 @@
       <c r="AJ21" s="1"/>
       <c r="AK21" s="1"/>
     </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>4</v>
       </c>
@@ -1936,7 +2077,7 @@
       </c>
       <c r="AK22" s="1"/>
     </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>19</v>
       </c>
@@ -1997,7 +2138,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>26</v>
       </c>
@@ -2046,7 +2187,7 @@
       <c r="AJ24" s="1"/>
       <c r="AK24" s="1"/>
     </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>48</v>
       </c>
@@ -2095,7 +2236,7 @@
       <c r="AJ25" s="1"/>
       <c r="AK25" s="1"/>
     </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>77</v>
       </c>
@@ -2148,295 +2289,851 @@
       <c r="AJ26" s="1"/>
       <c r="AK26" s="1"/>
     </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>52</v>
       </c>
-      <c r="H27">
-        <v>3</v>
-      </c>
-      <c r="Z27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="B27" s="1"/>
+      <c r="C27" s="1"/>
+      <c r="D27" s="1"/>
+      <c r="E27" s="1"/>
+      <c r="F27" s="1"/>
+      <c r="G27" s="1"/>
+      <c r="H27" s="1">
+        <v>3</v>
+      </c>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="1"/>
+      <c r="W27" s="1"/>
+      <c r="X27" s="1"/>
+      <c r="Y27" s="1"/>
+      <c r="Z27" s="1">
+        <v>3</v>
+      </c>
+      <c r="AA27" s="1"/>
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+      <c r="AE27" s="1"/>
+      <c r="AF27" s="1"/>
+      <c r="AG27" s="1"/>
+      <c r="AH27" s="1"/>
+      <c r="AI27" s="1"/>
+      <c r="AJ27" s="1"/>
+      <c r="AK27" s="1"/>
+      <c r="AL27" s="1"/>
+      <c r="AM27" s="1"/>
+      <c r="AN27" s="1"/>
+      <c r="AO27" s="1"/>
+      <c r="AP27" s="1"/>
+      <c r="AQ27" s="1"/>
+      <c r="AR27" s="1"/>
+      <c r="AS27" s="1"/>
+      <c r="AT27" s="1"/>
+    </row>
+    <row r="28" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A28">
         <v>54</v>
       </c>
-      <c r="H28">
-        <v>10</v>
-      </c>
-      <c r="M28">
-        <v>0.5</v>
-      </c>
-      <c r="O28">
-        <v>3</v>
-      </c>
-      <c r="Z28">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1">
+        <v>10</v>
+      </c>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1">
+        <v>3</v>
+      </c>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1">
+        <v>3</v>
+      </c>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+      <c r="AD28" s="1"/>
+      <c r="AE28" s="1"/>
+      <c r="AF28" s="1"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="1"/>
+      <c r="AI28" s="1"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="1"/>
+      <c r="AL28" s="1"/>
+      <c r="AM28" s="1"/>
+      <c r="AN28" s="1"/>
+      <c r="AO28" s="1"/>
+      <c r="AP28" s="1"/>
+      <c r="AQ28" s="1"/>
+      <c r="AR28" s="1"/>
+      <c r="AS28" s="1"/>
+      <c r="AT28" s="1"/>
+    </row>
+    <row r="29" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A29">
         <v>62</v>
       </c>
-      <c r="B29">
-        <v>3</v>
-      </c>
-      <c r="G29">
-        <v>0.5</v>
-      </c>
-      <c r="H29">
-        <v>3</v>
-      </c>
-      <c r="I29">
-        <v>10</v>
-      </c>
-      <c r="J29">
-        <v>0.5</v>
-      </c>
-      <c r="O29">
-        <v>3</v>
-      </c>
-      <c r="AC29">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="B29" s="1">
+        <v>3</v>
+      </c>
+      <c r="C29" s="1"/>
+      <c r="D29" s="1"/>
+      <c r="E29" s="1"/>
+      <c r="F29" s="1"/>
+      <c r="G29" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H29" s="1">
+        <v>3</v>
+      </c>
+      <c r="I29" s="1">
+        <v>10</v>
+      </c>
+      <c r="J29" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1">
+        <v>3</v>
+      </c>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="1"/>
+      <c r="W29" s="1"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="1"/>
+      <c r="Z29" s="1"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1">
+        <v>3</v>
+      </c>
+      <c r="AD29" s="1"/>
+      <c r="AE29" s="1"/>
+      <c r="AF29" s="1"/>
+      <c r="AG29" s="1"/>
+      <c r="AH29" s="1"/>
+      <c r="AI29" s="1"/>
+      <c r="AJ29" s="1"/>
+      <c r="AK29" s="1"/>
+      <c r="AL29" s="1"/>
+      <c r="AM29" s="1"/>
+      <c r="AN29" s="1"/>
+      <c r="AO29" s="1"/>
+      <c r="AP29" s="1"/>
+      <c r="AQ29" s="1"/>
+      <c r="AR29" s="1"/>
+      <c r="AS29" s="1"/>
+      <c r="AT29" s="1"/>
+    </row>
+    <row r="30" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A30">
         <v>98</v>
       </c>
-      <c r="B30">
-        <v>0.5</v>
-      </c>
-      <c r="H30">
-        <v>3</v>
-      </c>
-      <c r="AE30">
-        <v>0.5</v>
-      </c>
-      <c r="AL30">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="B30" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="D30" s="1"/>
+      <c r="E30" s="1"/>
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1">
+        <v>3</v>
+      </c>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+      <c r="R30" s="1"/>
+      <c r="S30" s="1"/>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="1"/>
+      <c r="W30" s="1"/>
+      <c r="X30" s="1"/>
+      <c r="Y30" s="1"/>
+      <c r="Z30" s="1"/>
+      <c r="AA30" s="1"/>
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+      <c r="AE30" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AF30" s="1"/>
+      <c r="AG30" s="1"/>
+      <c r="AH30" s="1"/>
+      <c r="AI30" s="1"/>
+      <c r="AJ30" s="1"/>
+      <c r="AK30" s="1"/>
+      <c r="AL30" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AM30" s="1"/>
+      <c r="AN30" s="1"/>
+      <c r="AO30" s="1"/>
+      <c r="AP30" s="1"/>
+      <c r="AQ30" s="1"/>
+      <c r="AR30" s="1"/>
+      <c r="AS30" s="1"/>
+      <c r="AT30" s="1"/>
+    </row>
+    <row r="31" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A31">
         <v>70</v>
       </c>
-      <c r="F31">
-        <v>3</v>
-      </c>
-      <c r="I31">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="B31" s="1"/>
+      <c r="C31" s="1"/>
+      <c r="D31" s="1"/>
+      <c r="E31" s="1"/>
+      <c r="F31" s="1">
+        <v>3</v>
+      </c>
+      <c r="G31" s="1"/>
+      <c r="H31" s="1"/>
+      <c r="I31" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+      <c r="R31" s="1"/>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+      <c r="W31" s="1"/>
+      <c r="X31" s="1"/>
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+      <c r="AG31" s="1"/>
+      <c r="AH31" s="1"/>
+      <c r="AI31" s="1"/>
+      <c r="AJ31" s="1"/>
+      <c r="AK31" s="1"/>
+      <c r="AL31" s="1"/>
+      <c r="AM31" s="1"/>
+      <c r="AN31" s="1"/>
+      <c r="AO31" s="1"/>
+      <c r="AP31" s="1"/>
+      <c r="AQ31" s="1"/>
+      <c r="AR31" s="1"/>
+      <c r="AS31" s="1"/>
+      <c r="AT31" s="1"/>
+    </row>
+    <row r="32" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A32">
         <v>86</v>
       </c>
-      <c r="H32">
-        <v>10</v>
-      </c>
-      <c r="I32">
-        <v>10</v>
-      </c>
-      <c r="J32">
-        <v>10</v>
-      </c>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1">
+        <v>10</v>
+      </c>
+      <c r="I32" s="1">
+        <v>10</v>
+      </c>
+      <c r="J32" s="1">
+        <v>10</v>
+      </c>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+      <c r="R32" s="1"/>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+      <c r="W32" s="1"/>
+      <c r="X32" s="1"/>
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
+      <c r="AA32" s="1"/>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+      <c r="AG32" s="1"/>
+      <c r="AH32" s="1"/>
+      <c r="AI32" s="1"/>
+      <c r="AJ32" s="1"/>
+      <c r="AK32" s="1"/>
+      <c r="AL32" s="1"/>
+      <c r="AM32" s="1"/>
+      <c r="AN32" s="1"/>
+      <c r="AO32" s="1"/>
+      <c r="AP32" s="1"/>
+      <c r="AQ32" s="1"/>
+      <c r="AR32" s="1"/>
+      <c r="AS32" s="1"/>
+      <c r="AT32" s="1"/>
     </row>
     <row r="33" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A33">
         <v>60</v>
       </c>
-      <c r="H33">
-        <v>0.5</v>
-      </c>
-      <c r="I33">
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I33" s="1">
         <v>20</v>
       </c>
-      <c r="J33">
-        <v>3</v>
-      </c>
-      <c r="AC33">
-        <v>0.5</v>
-      </c>
+      <c r="J33" s="1">
+        <v>3</v>
+      </c>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="1"/>
+      <c r="W33" s="1"/>
+      <c r="X33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AD33" s="1"/>
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+      <c r="AG33" s="1"/>
+      <c r="AH33" s="1"/>
+      <c r="AI33" s="1"/>
+      <c r="AJ33" s="1"/>
+      <c r="AK33" s="1"/>
+      <c r="AL33" s="1"/>
+      <c r="AM33" s="1"/>
+      <c r="AN33" s="1"/>
+      <c r="AO33" s="1"/>
+      <c r="AP33" s="1"/>
+      <c r="AQ33" s="1"/>
+      <c r="AR33" s="1"/>
+      <c r="AS33" s="1"/>
+      <c r="AT33" s="1"/>
     </row>
     <row r="34" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A34">
         <v>5</v>
       </c>
-      <c r="G34">
-        <v>0.5</v>
-      </c>
-      <c r="H34">
-        <v>0.5</v>
-      </c>
-      <c r="I34">
-        <v>3</v>
-      </c>
-      <c r="J34">
-        <v>0.5</v>
-      </c>
-      <c r="K34">
-        <v>0.5</v>
-      </c>
-      <c r="L34">
-        <v>3</v>
-      </c>
-      <c r="M34">
-        <v>3</v>
-      </c>
-      <c r="S34">
-        <v>3</v>
-      </c>
-      <c r="AC34">
-        <v>0.5</v>
-      </c>
-      <c r="AJ34">
+      <c r="B34" s="1"/>
+      <c r="C34" s="1"/>
+      <c r="D34" s="1"/>
+      <c r="E34" s="1"/>
+      <c r="F34" s="1"/>
+      <c r="G34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I34" s="1">
+        <v>3</v>
+      </c>
+      <c r="J34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="K34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="L34" s="1">
+        <v>3</v>
+      </c>
+      <c r="M34" s="1">
+        <v>3</v>
+      </c>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+      <c r="R34" s="1"/>
+      <c r="S34" s="1">
+        <v>3</v>
+      </c>
+      <c r="T34" s="1"/>
+      <c r="U34" s="1"/>
+      <c r="V34" s="1"/>
+      <c r="W34" s="1"/>
+      <c r="X34" s="1"/>
+      <c r="Y34" s="1"/>
+      <c r="Z34" s="1"/>
+      <c r="AA34" s="1"/>
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AD34" s="1"/>
+      <c r="AE34" s="1"/>
+      <c r="AF34" s="1"/>
+      <c r="AG34" s="1"/>
+      <c r="AH34" s="1"/>
+      <c r="AI34" s="1"/>
+      <c r="AJ34" s="1">
         <v>20</v>
       </c>
-      <c r="AL34">
-        <v>0.5</v>
-      </c>
+      <c r="AK34" s="1"/>
+      <c r="AL34" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AM34" s="1"/>
+      <c r="AN34" s="1"/>
+      <c r="AO34" s="1"/>
+      <c r="AP34" s="1"/>
+      <c r="AQ34" s="1"/>
+      <c r="AR34" s="1"/>
+      <c r="AS34" s="1"/>
+      <c r="AT34" s="1"/>
     </row>
     <row r="35" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A35">
         <v>81</v>
       </c>
-      <c r="F35">
-        <v>0.5</v>
-      </c>
-      <c r="L35">
-        <v>0.5</v>
-      </c>
-      <c r="M35">
-        <v>10</v>
-      </c>
-      <c r="U35">
-        <v>3</v>
-      </c>
-      <c r="V35">
-        <v>10</v>
-      </c>
-      <c r="AM35">
-        <v>0.5</v>
-      </c>
-      <c r="AN35">
-        <v>0.5</v>
-      </c>
-      <c r="AO35">
-        <v>3</v>
-      </c>
-      <c r="AP35">
-        <v>3</v>
-      </c>
-      <c r="AQ35">
-        <v>3</v>
-      </c>
-      <c r="AR35">
-        <v>0.5</v>
-      </c>
+      <c r="B35" s="1"/>
+      <c r="C35" s="1"/>
+      <c r="D35" s="1"/>
+      <c r="E35" s="1"/>
+      <c r="F35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="G35" s="1"/>
+      <c r="H35" s="1"/>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="M35" s="1">
+        <v>10</v>
+      </c>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1"/>
+      <c r="R35" s="1"/>
+      <c r="S35" s="1"/>
+      <c r="T35" s="1"/>
+      <c r="U35" s="1">
+        <v>3</v>
+      </c>
+      <c r="V35" s="1">
+        <v>10</v>
+      </c>
+      <c r="W35" s="1"/>
+      <c r="X35" s="1"/>
+      <c r="Y35" s="1"/>
+      <c r="Z35" s="1"/>
+      <c r="AA35" s="1"/>
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+      <c r="AD35" s="1"/>
+      <c r="AE35" s="1"/>
+      <c r="AF35" s="1"/>
+      <c r="AG35" s="1"/>
+      <c r="AH35" s="1"/>
+      <c r="AI35" s="1"/>
+      <c r="AJ35" s="1"/>
+      <c r="AK35" s="1"/>
+      <c r="AL35" s="1"/>
+      <c r="AM35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AN35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AO35" s="1">
+        <v>3</v>
+      </c>
+      <c r="AP35" s="1">
+        <v>3</v>
+      </c>
+      <c r="AQ35" s="1">
+        <v>3</v>
+      </c>
+      <c r="AR35" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AS35" s="1"/>
+      <c r="AT35" s="1"/>
     </row>
     <row r="36" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A36">
         <v>28</v>
       </c>
-      <c r="B36">
-        <v>0.5</v>
-      </c>
-      <c r="H36">
-        <v>3</v>
-      </c>
-      <c r="I36">
-        <v>3</v>
-      </c>
-      <c r="AH36">
-        <v>0.5</v>
-      </c>
+      <c r="B36" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="C36" s="1"/>
+      <c r="D36" s="1"/>
+      <c r="E36" s="1"/>
+      <c r="F36" s="1"/>
+      <c r="G36" s="1"/>
+      <c r="H36" s="1">
+        <v>3</v>
+      </c>
+      <c r="I36" s="1">
+        <v>3</v>
+      </c>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+      <c r="R36" s="1"/>
+      <c r="S36" s="1"/>
+      <c r="T36" s="1"/>
+      <c r="U36" s="1"/>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1"/>
+      <c r="X36" s="1"/>
+      <c r="Y36" s="1"/>
+      <c r="Z36" s="1"/>
+      <c r="AA36" s="1"/>
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+      <c r="AD36" s="1"/>
+      <c r="AE36" s="1"/>
+      <c r="AF36" s="1"/>
+      <c r="AG36" s="1"/>
+      <c r="AH36" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AI36" s="1"/>
+      <c r="AJ36" s="1"/>
+      <c r="AK36" s="1"/>
+      <c r="AL36" s="1"/>
+      <c r="AM36" s="1"/>
+      <c r="AN36" s="1"/>
+      <c r="AO36" s="1"/>
+      <c r="AP36" s="1"/>
+      <c r="AQ36" s="1"/>
+      <c r="AR36" s="1"/>
+      <c r="AS36" s="1"/>
+      <c r="AT36" s="1"/>
     </row>
     <row r="37" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A37">
         <v>36</v>
       </c>
-      <c r="I37">
-        <v>10</v>
-      </c>
-      <c r="S37">
-        <v>10</v>
-      </c>
-      <c r="U37">
-        <v>3</v>
-      </c>
+      <c r="B37" s="1"/>
+      <c r="C37" s="1"/>
+      <c r="D37" s="1"/>
+      <c r="E37" s="1"/>
+      <c r="F37" s="1"/>
+      <c r="G37" s="1"/>
+      <c r="H37" s="1"/>
+      <c r="I37" s="1">
+        <v>10</v>
+      </c>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
+      <c r="R37" s="1"/>
+      <c r="S37" s="1">
+        <v>10</v>
+      </c>
+      <c r="T37" s="1"/>
+      <c r="U37" s="1">
+        <v>3</v>
+      </c>
+      <c r="V37" s="1"/>
+      <c r="W37" s="1"/>
+      <c r="X37" s="1"/>
+      <c r="Y37" s="1"/>
+      <c r="Z37" s="1"/>
+      <c r="AA37" s="1"/>
+      <c r="AB37" s="1"/>
+      <c r="AC37" s="1"/>
+      <c r="AD37" s="1"/>
+      <c r="AE37" s="1"/>
+      <c r="AF37" s="1"/>
+      <c r="AG37" s="1"/>
+      <c r="AH37" s="1"/>
+      <c r="AI37" s="1"/>
+      <c r="AJ37" s="1"/>
+      <c r="AK37" s="1"/>
+      <c r="AL37" s="1"/>
+      <c r="AM37" s="1"/>
+      <c r="AN37" s="1"/>
+      <c r="AO37" s="1"/>
+      <c r="AP37" s="1"/>
+      <c r="AQ37" s="1"/>
+      <c r="AR37" s="1"/>
+      <c r="AS37" s="1"/>
+      <c r="AT37" s="1"/>
     </row>
     <row r="38" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A38">
         <v>58</v>
       </c>
-      <c r="B38">
-        <v>3</v>
-      </c>
-      <c r="I38">
-        <v>3</v>
-      </c>
-      <c r="L38">
-        <v>10</v>
-      </c>
-      <c r="M38">
-        <v>3</v>
-      </c>
-      <c r="AI38">
-        <v>3</v>
-      </c>
+      <c r="B38" s="1">
+        <v>3</v>
+      </c>
+      <c r="C38" s="1"/>
+      <c r="D38" s="1"/>
+      <c r="E38" s="1"/>
+      <c r="F38" s="1"/>
+      <c r="G38" s="1"/>
+      <c r="H38" s="1"/>
+      <c r="I38" s="1">
+        <v>3</v>
+      </c>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1">
+        <v>10</v>
+      </c>
+      <c r="M38" s="1">
+        <v>3</v>
+      </c>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="1"/>
+      <c r="R38" s="1"/>
+      <c r="S38" s="1"/>
+      <c r="T38" s="1"/>
+      <c r="U38" s="1"/>
+      <c r="V38" s="1"/>
+      <c r="W38" s="1"/>
+      <c r="X38" s="1"/>
+      <c r="Y38" s="1"/>
+      <c r="Z38" s="1"/>
+      <c r="AA38" s="1"/>
+      <c r="AB38" s="1"/>
+      <c r="AC38" s="1"/>
+      <c r="AD38" s="1"/>
+      <c r="AE38" s="1"/>
+      <c r="AF38" s="1"/>
+      <c r="AG38" s="1"/>
+      <c r="AH38" s="1"/>
+      <c r="AI38" s="1">
+        <v>3</v>
+      </c>
+      <c r="AJ38" s="1"/>
+      <c r="AK38" s="1"/>
+      <c r="AL38" s="1"/>
+      <c r="AM38" s="1"/>
+      <c r="AN38" s="1"/>
+      <c r="AO38" s="1"/>
+      <c r="AP38" s="1"/>
+      <c r="AQ38" s="1"/>
+      <c r="AR38" s="1"/>
+      <c r="AS38" s="1"/>
+      <c r="AT38" s="1"/>
     </row>
     <row r="39" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A39">
         <v>73</v>
       </c>
-      <c r="F39">
-        <v>10</v>
-      </c>
-      <c r="H39">
-        <v>10</v>
-      </c>
-      <c r="M39">
+      <c r="B39" s="1"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="1"/>
+      <c r="F39" s="1">
+        <v>10</v>
+      </c>
+      <c r="G39" s="1"/>
+      <c r="H39" s="1">
+        <v>10</v>
+      </c>
+      <c r="I39" s="1"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1">
         <v>30</v>
       </c>
-      <c r="X39">
-        <v>10</v>
-      </c>
-      <c r="AL39">
-        <v>10</v>
-      </c>
-      <c r="AO39">
-        <v>3</v>
-      </c>
-      <c r="AS39">
-        <v>3</v>
-      </c>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="1"/>
+      <c r="R39" s="1"/>
+      <c r="S39" s="1"/>
+      <c r="T39" s="1"/>
+      <c r="U39" s="1"/>
+      <c r="V39" s="1"/>
+      <c r="W39" s="1"/>
+      <c r="X39" s="1">
+        <v>10</v>
+      </c>
+      <c r="Y39" s="1"/>
+      <c r="Z39" s="1"/>
+      <c r="AA39" s="1"/>
+      <c r="AB39" s="1"/>
+      <c r="AC39" s="1"/>
+      <c r="AD39" s="1"/>
+      <c r="AE39" s="1"/>
+      <c r="AF39" s="1"/>
+      <c r="AG39" s="1"/>
+      <c r="AH39" s="1"/>
+      <c r="AI39" s="1"/>
+      <c r="AJ39" s="1"/>
+      <c r="AK39" s="1"/>
+      <c r="AL39" s="1">
+        <v>10</v>
+      </c>
+      <c r="AM39" s="1"/>
+      <c r="AN39" s="1"/>
+      <c r="AO39" s="1">
+        <v>3</v>
+      </c>
+      <c r="AP39" s="1"/>
+      <c r="AQ39" s="1"/>
+      <c r="AR39" s="1"/>
+      <c r="AS39" s="1">
+        <v>3</v>
+      </c>
+      <c r="AT39" s="1"/>
     </row>
     <row r="40" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A40">
         <v>75</v>
       </c>
-      <c r="F40">
-        <v>10</v>
-      </c>
-      <c r="H40">
-        <v>0.5</v>
-      </c>
-      <c r="I40">
-        <v>0.5</v>
-      </c>
-      <c r="O40">
-        <v>0.5</v>
-      </c>
-      <c r="U40">
-        <v>0.5</v>
-      </c>
-      <c r="AC40">
-        <v>0.5</v>
-      </c>
-      <c r="AT40">
+      <c r="B40" s="1"/>
+      <c r="C40" s="1"/>
+      <c r="D40" s="1"/>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1">
+        <v>10</v>
+      </c>
+      <c r="G40" s="1"/>
+      <c r="H40" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I40" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="P40" s="1"/>
+      <c r="Q40" s="1"/>
+      <c r="R40" s="1"/>
+      <c r="S40" s="1"/>
+      <c r="T40" s="1"/>
+      <c r="U40" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="V40" s="1"/>
+      <c r="W40" s="1"/>
+      <c r="X40" s="1"/>
+      <c r="Y40" s="1"/>
+      <c r="Z40" s="1"/>
+      <c r="AA40" s="1"/>
+      <c r="AB40" s="1"/>
+      <c r="AC40" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AD40" s="1"/>
+      <c r="AE40" s="1"/>
+      <c r="AF40" s="1"/>
+      <c r="AG40" s="1"/>
+      <c r="AH40" s="1"/>
+      <c r="AI40" s="1"/>
+      <c r="AJ40" s="1"/>
+      <c r="AK40" s="1"/>
+      <c r="AL40" s="1"/>
+      <c r="AM40" s="1"/>
+      <c r="AN40" s="1"/>
+      <c r="AO40" s="1"/>
+      <c r="AP40" s="1"/>
+      <c r="AQ40" s="1"/>
+      <c r="AR40" s="1"/>
+      <c r="AS40" s="1"/>
+      <c r="AT40" s="1">
         <v>0.5</v>
       </c>
     </row>
@@ -2444,190 +3141,1027 @@
       <c r="A41">
         <v>42</v>
       </c>
-      <c r="F41">
-        <v>3</v>
-      </c>
-      <c r="H41">
-        <v>10</v>
-      </c>
-      <c r="M41">
-        <v>3</v>
-      </c>
-      <c r="R41">
-        <v>3</v>
-      </c>
-      <c r="AL41">
-        <v>3</v>
-      </c>
-      <c r="AN41">
-        <v>0.5</v>
-      </c>
-      <c r="AS41">
-        <v>10</v>
-      </c>
+      <c r="B41" s="1"/>
+      <c r="C41" s="1"/>
+      <c r="D41" s="1"/>
+      <c r="E41" s="1"/>
+      <c r="F41" s="1">
+        <v>3</v>
+      </c>
+      <c r="G41" s="1"/>
+      <c r="H41" s="1">
+        <v>10</v>
+      </c>
+      <c r="I41" s="1"/>
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1">
+        <v>3</v>
+      </c>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
+      <c r="P41" s="1"/>
+      <c r="Q41" s="1"/>
+      <c r="R41" s="1">
+        <v>3</v>
+      </c>
+      <c r="S41" s="1"/>
+      <c r="T41" s="1"/>
+      <c r="U41" s="1"/>
+      <c r="V41" s="1"/>
+      <c r="W41" s="1"/>
+      <c r="X41" s="1"/>
+      <c r="Y41" s="1"/>
+      <c r="Z41" s="1"/>
+      <c r="AA41" s="1"/>
+      <c r="AB41" s="1"/>
+      <c r="AC41" s="1"/>
+      <c r="AD41" s="1"/>
+      <c r="AE41" s="1"/>
+      <c r="AF41" s="1"/>
+      <c r="AG41" s="1"/>
+      <c r="AH41" s="1"/>
+      <c r="AI41" s="1"/>
+      <c r="AJ41" s="1"/>
+      <c r="AK41" s="1"/>
+      <c r="AL41" s="1">
+        <v>3</v>
+      </c>
+      <c r="AM41" s="1"/>
+      <c r="AN41" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AO41" s="1"/>
+      <c r="AP41" s="1"/>
+      <c r="AQ41" s="1"/>
+      <c r="AR41" s="1"/>
+      <c r="AS41" s="1">
+        <v>10</v>
+      </c>
+      <c r="AT41" s="1"/>
     </row>
     <row r="42" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A42">
         <v>6</v>
       </c>
-      <c r="F42">
-        <v>10</v>
-      </c>
-      <c r="H42">
-        <v>3</v>
-      </c>
+      <c r="B42" s="1"/>
+      <c r="C42" s="1"/>
+      <c r="D42" s="1"/>
+      <c r="E42" s="1"/>
+      <c r="F42" s="1">
+        <v>10</v>
+      </c>
+      <c r="G42" s="1"/>
+      <c r="H42" s="1">
+        <v>3</v>
+      </c>
+      <c r="I42" s="1"/>
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
+      <c r="P42" s="1"/>
+      <c r="Q42" s="1"/>
+      <c r="R42" s="1"/>
+      <c r="S42" s="1"/>
+      <c r="T42" s="1"/>
+      <c r="U42" s="1"/>
+      <c r="V42" s="1"/>
+      <c r="W42" s="1"/>
+      <c r="X42" s="1"/>
+      <c r="Y42" s="1"/>
+      <c r="Z42" s="1"/>
+      <c r="AA42" s="1"/>
+      <c r="AB42" s="1"/>
+      <c r="AC42" s="1"/>
+      <c r="AD42" s="1"/>
+      <c r="AE42" s="1"/>
+      <c r="AF42" s="1"/>
+      <c r="AG42" s="1"/>
+      <c r="AH42" s="1"/>
+      <c r="AI42" s="1"/>
+      <c r="AJ42" s="1"/>
+      <c r="AK42" s="1"/>
+      <c r="AL42" s="1"/>
+      <c r="AM42" s="1"/>
+      <c r="AN42" s="1"/>
+      <c r="AO42" s="1"/>
+      <c r="AP42" s="1"/>
+      <c r="AQ42" s="1"/>
+      <c r="AR42" s="1"/>
+      <c r="AS42" s="1"/>
+      <c r="AT42" s="1"/>
     </row>
     <row r="43" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A43">
         <v>1</v>
       </c>
-      <c r="H43">
-        <v>0.5</v>
-      </c>
-      <c r="I43">
+      <c r="B43" s="1"/>
+      <c r="C43" s="1"/>
+      <c r="D43" s="1"/>
+      <c r="E43" s="1"/>
+      <c r="F43" s="1"/>
+      <c r="G43" s="1"/>
+      <c r="H43" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I43" s="1">
         <v>30</v>
       </c>
-      <c r="AC43">
-        <v>3</v>
-      </c>
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
+      <c r="P43" s="1"/>
+      <c r="Q43" s="1"/>
+      <c r="R43" s="1"/>
+      <c r="S43" s="1"/>
+      <c r="T43" s="1"/>
+      <c r="U43" s="1"/>
+      <c r="V43" s="1"/>
+      <c r="W43" s="1"/>
+      <c r="X43" s="1"/>
+      <c r="Y43" s="1"/>
+      <c r="Z43" s="1"/>
+      <c r="AA43" s="1"/>
+      <c r="AB43" s="1"/>
+      <c r="AC43" s="1">
+        <v>3</v>
+      </c>
+      <c r="AD43" s="1"/>
+      <c r="AE43" s="1"/>
+      <c r="AF43" s="1"/>
+      <c r="AG43" s="1"/>
+      <c r="AH43" s="1"/>
+      <c r="AI43" s="1"/>
+      <c r="AJ43" s="1"/>
+      <c r="AK43" s="1"/>
+      <c r="AL43" s="1"/>
+      <c r="AM43" s="1"/>
+      <c r="AN43" s="1"/>
+      <c r="AO43" s="1"/>
+      <c r="AP43" s="1"/>
+      <c r="AQ43" s="1"/>
+      <c r="AR43" s="1"/>
+      <c r="AS43" s="1"/>
+      <c r="AT43" s="1"/>
     </row>
     <row r="44" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A44">
         <v>100</v>
       </c>
-      <c r="H44">
-        <v>3</v>
-      </c>
-      <c r="I44">
-        <v>0.5</v>
-      </c>
-      <c r="J44">
-        <v>3</v>
-      </c>
-      <c r="Q44">
-        <v>0.5</v>
-      </c>
-      <c r="R44">
-        <v>0.5</v>
-      </c>
-      <c r="Z44">
-        <v>10</v>
-      </c>
+      <c r="B44" s="1"/>
+      <c r="C44" s="1"/>
+      <c r="D44" s="1"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="1"/>
+      <c r="G44" s="1"/>
+      <c r="H44" s="1">
+        <v>3</v>
+      </c>
+      <c r="I44" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J44" s="1">
+        <v>3</v>
+      </c>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
+      <c r="P44" s="1"/>
+      <c r="Q44" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="R44" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="S44" s="1"/>
+      <c r="T44" s="1"/>
+      <c r="U44" s="1"/>
+      <c r="V44" s="1"/>
+      <c r="W44" s="1"/>
+      <c r="X44" s="1"/>
+      <c r="Y44" s="1"/>
+      <c r="Z44" s="1">
+        <v>10</v>
+      </c>
+      <c r="AA44" s="1"/>
+      <c r="AB44" s="1"/>
+      <c r="AC44" s="1"/>
+      <c r="AD44" s="1"/>
+      <c r="AE44" s="1"/>
+      <c r="AF44" s="1"/>
+      <c r="AG44" s="1"/>
+      <c r="AH44" s="1"/>
+      <c r="AI44" s="1"/>
+      <c r="AJ44" s="1"/>
+      <c r="AK44" s="1"/>
+      <c r="AL44" s="1"/>
+      <c r="AM44" s="1"/>
+      <c r="AN44" s="1"/>
+      <c r="AO44" s="1"/>
+      <c r="AP44" s="1"/>
+      <c r="AQ44" s="1"/>
+      <c r="AR44" s="1"/>
+      <c r="AS44" s="1"/>
+      <c r="AT44" s="1"/>
     </row>
     <row r="45" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A45">
         <v>10</v>
       </c>
-      <c r="I45">
+      <c r="B45" s="1"/>
+      <c r="C45" s="1"/>
+      <c r="D45" s="1"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="1"/>
+      <c r="G45" s="1"/>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1">
         <v>20</v>
       </c>
-      <c r="J45">
+      <c r="J45" s="1">
         <v>20</v>
       </c>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
+      <c r="P45" s="1"/>
+      <c r="Q45" s="1"/>
+      <c r="R45" s="1"/>
+      <c r="S45" s="1"/>
+      <c r="T45" s="1"/>
+      <c r="U45" s="1"/>
+      <c r="V45" s="1"/>
+      <c r="W45" s="1"/>
+      <c r="X45" s="1"/>
+      <c r="Y45" s="1"/>
+      <c r="Z45" s="1"/>
+      <c r="AA45" s="1"/>
+      <c r="AB45" s="1"/>
+      <c r="AC45" s="1"/>
+      <c r="AD45" s="1"/>
+      <c r="AE45" s="1"/>
+      <c r="AF45" s="1"/>
+      <c r="AG45" s="1"/>
+      <c r="AH45" s="1"/>
+      <c r="AI45" s="1"/>
+      <c r="AJ45" s="1"/>
+      <c r="AK45" s="1"/>
+      <c r="AL45" s="1"/>
+      <c r="AM45" s="1"/>
+      <c r="AN45" s="1"/>
+      <c r="AO45" s="1"/>
+      <c r="AP45" s="1"/>
+      <c r="AQ45" s="1"/>
+      <c r="AR45" s="1"/>
+      <c r="AS45" s="1"/>
+      <c r="AT45" s="1"/>
     </row>
     <row r="46" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A46">
         <v>79</v>
       </c>
-      <c r="H46">
-        <v>10</v>
-      </c>
-      <c r="I46">
-        <v>10</v>
-      </c>
+      <c r="B46" s="1"/>
+      <c r="C46" s="1"/>
+      <c r="D46" s="1"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="1"/>
+      <c r="G46" s="1"/>
+      <c r="H46" s="1">
+        <v>10</v>
+      </c>
+      <c r="I46" s="1">
+        <v>10</v>
+      </c>
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1"/>
+      <c r="P46" s="1"/>
+      <c r="Q46" s="1"/>
+      <c r="R46" s="1"/>
+      <c r="S46" s="1"/>
+      <c r="T46" s="1"/>
+      <c r="U46" s="1"/>
+      <c r="V46" s="1"/>
+      <c r="W46" s="1"/>
+      <c r="X46" s="1"/>
+      <c r="Y46" s="1"/>
+      <c r="Z46" s="1"/>
+      <c r="AA46" s="1"/>
+      <c r="AB46" s="1"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1"/>
+      <c r="AE46" s="1"/>
+      <c r="AF46" s="1"/>
+      <c r="AG46" s="1"/>
+      <c r="AH46" s="1"/>
+      <c r="AI46" s="1"/>
+      <c r="AJ46" s="1"/>
+      <c r="AK46" s="1"/>
+      <c r="AL46" s="1"/>
+      <c r="AM46" s="1"/>
+      <c r="AN46" s="1"/>
+      <c r="AO46" s="1"/>
+      <c r="AP46" s="1"/>
+      <c r="AQ46" s="1"/>
+      <c r="AR46" s="1"/>
+      <c r="AS46" s="1"/>
+      <c r="AT46" s="1"/>
     </row>
     <row r="47" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A47">
         <v>29</v>
       </c>
-      <c r="B47">
+      <c r="B47" s="1">
         <v>20</v>
       </c>
-      <c r="H47">
-        <v>3</v>
-      </c>
-      <c r="X47">
-        <v>3</v>
-      </c>
-      <c r="AL47">
-        <v>10</v>
-      </c>
+      <c r="C47" s="1"/>
+      <c r="D47" s="1"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="1"/>
+      <c r="G47" s="1"/>
+      <c r="H47" s="1">
+        <v>3</v>
+      </c>
+      <c r="I47" s="1"/>
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1"/>
+      <c r="P47" s="1"/>
+      <c r="Q47" s="1"/>
+      <c r="R47" s="1"/>
+      <c r="S47" s="1"/>
+      <c r="T47" s="1"/>
+      <c r="U47" s="1"/>
+      <c r="V47" s="1"/>
+      <c r="W47" s="1"/>
+      <c r="X47" s="1">
+        <v>3</v>
+      </c>
+      <c r="Y47" s="1"/>
+      <c r="Z47" s="1"/>
+      <c r="AA47" s="1"/>
+      <c r="AB47" s="1"/>
+      <c r="AC47" s="1"/>
+      <c r="AD47" s="1"/>
+      <c r="AE47" s="1"/>
+      <c r="AF47" s="1"/>
+      <c r="AG47" s="1"/>
+      <c r="AH47" s="1"/>
+      <c r="AI47" s="1"/>
+      <c r="AJ47" s="1"/>
+      <c r="AK47" s="1"/>
+      <c r="AL47" s="1">
+        <v>10</v>
+      </c>
+      <c r="AM47" s="1"/>
+      <c r="AN47" s="1"/>
+      <c r="AO47" s="1"/>
+      <c r="AP47" s="1"/>
+      <c r="AQ47" s="1"/>
+      <c r="AR47" s="1"/>
+      <c r="AS47" s="1"/>
+      <c r="AT47" s="1"/>
     </row>
     <row r="48" spans="1:46" x14ac:dyDescent="0.2">
       <c r="A48">
         <v>16</v>
       </c>
-      <c r="B48">
-        <v>3</v>
-      </c>
-      <c r="H48">
-        <v>3</v>
-      </c>
-      <c r="I48">
-        <v>10</v>
-      </c>
-      <c r="Q48">
-        <v>3</v>
-      </c>
-      <c r="S48">
-        <v>0.5</v>
-      </c>
-      <c r="AI48">
-        <v>0.5</v>
-      </c>
-      <c r="AL48">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="B48" s="1">
+        <v>3</v>
+      </c>
+      <c r="C48" s="1"/>
+      <c r="D48" s="1"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="1"/>
+      <c r="G48" s="1"/>
+      <c r="H48" s="1">
+        <v>3</v>
+      </c>
+      <c r="I48" s="1">
+        <v>10</v>
+      </c>
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1"/>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="1">
+        <v>3</v>
+      </c>
+      <c r="R48" s="1"/>
+      <c r="S48" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="T48" s="1"/>
+      <c r="U48" s="1"/>
+      <c r="V48" s="1"/>
+      <c r="W48" s="1"/>
+      <c r="X48" s="1"/>
+      <c r="Y48" s="1"/>
+      <c r="Z48" s="1"/>
+      <c r="AA48" s="1"/>
+      <c r="AB48" s="1"/>
+      <c r="AC48" s="1"/>
+      <c r="AD48" s="1"/>
+      <c r="AE48" s="1"/>
+      <c r="AF48" s="1"/>
+      <c r="AG48" s="1"/>
+      <c r="AH48" s="1"/>
+      <c r="AI48" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AJ48" s="1"/>
+      <c r="AK48" s="1"/>
+      <c r="AL48" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="AM48" s="1"/>
+      <c r="AN48" s="1"/>
+      <c r="AO48" s="1"/>
+      <c r="AP48" s="1"/>
+      <c r="AQ48" s="1"/>
+      <c r="AR48" s="1"/>
+      <c r="AS48" s="1"/>
+      <c r="AT48" s="1"/>
+    </row>
+    <row r="49" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A49">
         <v>23</v>
       </c>
-      <c r="G49">
-        <v>3</v>
-      </c>
-      <c r="H49">
-        <v>10</v>
-      </c>
-      <c r="I49">
-        <v>0.5</v>
-      </c>
-      <c r="J49">
-        <v>3</v>
-      </c>
-      <c r="M49">
+      <c r="B49" s="1"/>
+      <c r="C49" s="1"/>
+      <c r="D49" s="1"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="1"/>
+      <c r="G49" s="1">
+        <v>3</v>
+      </c>
+      <c r="H49" s="1">
+        <v>10</v>
+      </c>
+      <c r="I49" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="J49" s="1">
+        <v>3</v>
+      </c>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1">
         <v>20</v>
       </c>
-      <c r="O49">
-        <v>3</v>
-      </c>
-      <c r="U49">
-        <v>3</v>
-      </c>
-      <c r="X49">
-        <v>0.5</v>
-      </c>
-      <c r="Z49">
+      <c r="N49" s="1"/>
+      <c r="O49" s="1">
+        <v>3</v>
+      </c>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="1"/>
+      <c r="R49" s="1"/>
+      <c r="S49" s="1"/>
+      <c r="T49" s="1"/>
+      <c r="U49" s="1">
+        <v>3</v>
+      </c>
+      <c r="V49" s="1"/>
+      <c r="W49" s="1"/>
+      <c r="X49" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="Y49" s="1"/>
+      <c r="Z49" s="1">
         <v>30</v>
       </c>
-      <c r="AG49">
-        <v>10</v>
-      </c>
-      <c r="AJ49">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AA49" s="1"/>
+      <c r="AB49" s="1"/>
+      <c r="AC49" s="1"/>
+      <c r="AD49" s="1"/>
+      <c r="AE49" s="1"/>
+      <c r="AF49" s="1"/>
+      <c r="AG49" s="1">
+        <v>10</v>
+      </c>
+      <c r="AH49" s="1"/>
+      <c r="AI49" s="1"/>
+      <c r="AJ49" s="1">
+        <v>3</v>
+      </c>
+      <c r="AK49" s="1"/>
+      <c r="AL49" s="1"/>
+      <c r="AM49" s="1"/>
+      <c r="AN49" s="1"/>
+      <c r="AO49" s="1"/>
+      <c r="AP49" s="1"/>
+      <c r="AQ49" s="1"/>
+      <c r="AR49" s="1"/>
+      <c r="AS49" s="1"/>
+      <c r="AT49" s="1"/>
+    </row>
+    <row r="50" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A50">
         <v>12</v>
       </c>
-      <c r="G50">
-        <v>0.5</v>
-      </c>
-      <c r="H50">
-        <v>0.5</v>
-      </c>
-      <c r="AN50">
+      <c r="B50" s="1"/>
+      <c r="C50" s="1"/>
+      <c r="D50" s="1"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="1"/>
+      <c r="G50" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="H50" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="I50" s="1"/>
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="1"/>
+      <c r="R50" s="1"/>
+      <c r="S50" s="1"/>
+      <c r="T50" s="1"/>
+      <c r="U50" s="1"/>
+      <c r="V50" s="1"/>
+      <c r="W50" s="1"/>
+      <c r="X50" s="1"/>
+      <c r="Y50" s="1"/>
+      <c r="Z50" s="1"/>
+      <c r="AA50" s="1"/>
+      <c r="AB50" s="1"/>
+      <c r="AC50" s="1"/>
+      <c r="AD50" s="1"/>
+      <c r="AE50" s="1"/>
+      <c r="AF50" s="1"/>
+      <c r="AG50" s="1"/>
+      <c r="AH50" s="1"/>
+      <c r="AI50" s="1"/>
+      <c r="AJ50" s="1"/>
+      <c r="AK50" s="1"/>
+      <c r="AL50" s="1"/>
+      <c r="AM50" s="1"/>
+      <c r="AN50" s="1">
+        <v>3</v>
+      </c>
+      <c r="AO50" s="1"/>
+      <c r="AP50" s="1"/>
+      <c r="AQ50" s="1"/>
+      <c r="AR50" s="1"/>
+      <c r="AS50" s="1"/>
+      <c r="AT50" s="1"/>
+    </row>
+    <row r="51" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>45</v>
+      </c>
+      <c r="B51">
+        <v>0.5</v>
+      </c>
+      <c r="I51">
+        <v>0.5</v>
+      </c>
+      <c r="L51">
+        <v>3</v>
+      </c>
+      <c r="AU51">
+        <v>0.5</v>
+      </c>
+      <c r="AV51">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="52" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>48</v>
+      </c>
+      <c r="H52">
+        <v>3</v>
+      </c>
+      <c r="U52">
+        <v>3</v>
+      </c>
+      <c r="Z52">
+        <v>3</v>
+      </c>
+      <c r="AJ52">
+        <v>0.5</v>
+      </c>
+      <c r="AW52">
+        <v>3</v>
+      </c>
+      <c r="AY52">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>50</v>
+      </c>
+      <c r="I53">
+        <v>20</v>
+      </c>
+      <c r="AI53">
+        <v>0.5</v>
+      </c>
+      <c r="AX53">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="54" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>52</v>
+      </c>
+      <c r="C54">
+        <v>10</v>
+      </c>
+      <c r="G54">
+        <v>0.5</v>
+      </c>
+      <c r="H54">
+        <v>3</v>
+      </c>
+      <c r="J54">
+        <v>0.5</v>
+      </c>
+      <c r="M54">
+        <v>3</v>
+      </c>
+      <c r="R54">
+        <v>0.5</v>
+      </c>
+      <c r="X54">
+        <v>0.5</v>
+      </c>
+      <c r="Z54">
+        <v>3</v>
+      </c>
+      <c r="AN54">
+        <v>0.5</v>
+      </c>
+      <c r="AZ54">
+        <v>3</v>
+      </c>
+      <c r="BA54">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>56</v>
+      </c>
+      <c r="U55">
+        <v>0.5</v>
+      </c>
+      <c r="AB55">
+        <v>10</v>
+      </c>
+      <c r="BB55">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="56" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>58</v>
+      </c>
+      <c r="F56">
+        <v>10</v>
+      </c>
+      <c r="M56">
+        <v>10</v>
+      </c>
+      <c r="AQ56">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="57" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>59</v>
+      </c>
+      <c r="F57">
+        <v>0.5</v>
+      </c>
+      <c r="I57">
+        <v>3</v>
+      </c>
+      <c r="L57">
+        <v>0.5</v>
+      </c>
+      <c r="AE57">
+        <v>0.5</v>
+      </c>
+      <c r="AW57">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="58" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="59" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>61</v>
+      </c>
+      <c r="F59">
+        <v>40</v>
+      </c>
+      <c r="AT59">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="60" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>62</v>
+      </c>
+      <c r="I60">
+        <v>10</v>
+      </c>
+      <c r="L60">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="61" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>63</v>
+      </c>
+      <c r="F61">
+        <v>3</v>
+      </c>
+      <c r="Z61">
+        <v>3</v>
+      </c>
+      <c r="AC61">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="62" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>64</v>
+      </c>
+      <c r="F62">
+        <v>10</v>
+      </c>
+      <c r="I62">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="63" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A63" t="s">
+        <v>65</v>
+      </c>
+      <c r="I63">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="64" spans="1:54" x14ac:dyDescent="0.2">
+      <c r="A64" t="s">
+        <v>66</v>
+      </c>
+      <c r="H64">
+        <v>0.5</v>
+      </c>
+      <c r="I64">
+        <v>3</v>
+      </c>
+      <c r="L64">
+        <v>10</v>
+      </c>
+      <c r="M64">
+        <v>0.5</v>
+      </c>
+      <c r="U64">
+        <v>3</v>
+      </c>
+      <c r="Y64">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
+        <v>67</v>
+      </c>
+      <c r="M65">
+        <v>10</v>
+      </c>
+      <c r="AZ65">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>68</v>
+      </c>
+      <c r="F66">
+        <v>10</v>
+      </c>
+      <c r="H66">
+        <v>3</v>
+      </c>
+      <c r="U66">
+        <v>20</v>
+      </c>
+      <c r="AT66">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>69</v>
+      </c>
+      <c r="B67">
+        <v>0.5</v>
+      </c>
+      <c r="H67">
+        <v>0.5</v>
+      </c>
+      <c r="I67">
+        <v>3</v>
+      </c>
+      <c r="R67">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>70</v>
+      </c>
+      <c r="D68">
+        <v>3</v>
+      </c>
+      <c r="M68">
+        <v>3</v>
+      </c>
+      <c r="V68">
+        <v>3</v>
+      </c>
+      <c r="W68">
+        <v>0.5</v>
+      </c>
+      <c r="Z68">
+        <v>0.5</v>
+      </c>
+      <c r="BC68">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="69" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>72</v>
+      </c>
+      <c r="F69">
+        <v>3</v>
+      </c>
+      <c r="I69">
+        <v>10</v>
+      </c>
+      <c r="K69">
+        <v>0.5</v>
+      </c>
+      <c r="AK69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>73</v>
+      </c>
+      <c r="M70">
+        <v>0.5</v>
+      </c>
+      <c r="S70">
+        <v>0.5</v>
+      </c>
+      <c r="U70">
+        <v>3</v>
+      </c>
+      <c r="AE70">
+        <v>3</v>
+      </c>
+      <c r="AU70">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>74</v>
+      </c>
+      <c r="I71">
+        <v>20</v>
+      </c>
+      <c r="BC71">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="72" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A72" t="s">
+        <v>75</v>
+      </c>
+      <c r="I72">
+        <v>10</v>
+      </c>
+      <c r="O72">
+        <v>0.5</v>
+      </c>
+      <c r="U72">
+        <v>0.5</v>
+      </c>
+      <c r="AU72">
+        <v>0.5</v>
+      </c>
+      <c r="AX72">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>76</v>
+      </c>
+      <c r="G73">
+        <v>0.5</v>
+      </c>
+      <c r="H73">
+        <v>0.5</v>
+      </c>
+      <c r="I73">
+        <v>3</v>
+      </c>
+      <c r="J73">
+        <v>0.5</v>
+      </c>
+      <c r="O73">
+        <v>3</v>
+      </c>
+      <c r="R73">
+        <v>0.5</v>
+      </c>
+      <c r="U73">
+        <v>3</v>
+      </c>
+      <c r="AC73">
+        <v>0.5</v>
+      </c>
+      <c r="AE73">
+        <v>0.5</v>
+      </c>
+      <c r="AR73">
+        <v>10</v>
+      </c>
+      <c r="BD73">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="74" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A74" t="s">
+        <v>78</v>
+      </c>
+      <c r="F74">
+        <v>0.5</v>
+      </c>
+      <c r="H74">
+        <v>0.5</v>
+      </c>
+      <c r="I74">
+        <v>10</v>
+      </c>
+      <c r="L74">
+        <v>0.5</v>
+      </c>
+      <c r="O74">
+        <v>3</v>
+      </c>
+      <c r="S74">
+        <v>0.5</v>
+      </c>
+      <c r="BE74">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="75" spans="1:57" x14ac:dyDescent="0.2">
+      <c r="A75" t="s">
+        <v>80</v>
+      </c>
+      <c r="I75">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
entered some more data
</commit_message>
<xml_diff>
--- a/data/community_fall2026.xlsx
+++ b/data/community_fall2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fernbromley/Desktop/AVCA_BANWR/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{792B1686-1F6D-C343-ADC4-DAB68D1987DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D023E04-BD4C-8943-BBBC-0497B43BCAD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="17200" xr2:uid="{7D6DEC84-1D80-5044-AEB0-AE046E367DDB}"/>
   </bookViews>
@@ -45,6 +45,8 @@
     <author>tc={CAF2C8A5-7E2B-F541-9DFB-700ACA44C592}</author>
     <author>tc={AB0CE727-E125-8144-8002-E2E433E4C919}</author>
     <author>tc={9D1C2B35-25B3-DE40-B60B-62E13F57E42C}</author>
+    <author>tc={239EA25F-C042-224C-8583-7C08AAF67E1F}</author>
+    <author>tc={F5E67526-0680-034D-8892-EF4DAD13EEE1}</author>
     <author>tc={841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}</author>
   </authors>
   <commentList>
@@ -80,7 +82,23 @@
     Atriplex elegans ("unk ama" on plot 98, by the road)</t>
       </text>
     </comment>
-    <comment ref="H7" authorId="4" shapeId="0" xr:uid="{841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}">
+    <comment ref="AU1" authorId="4" shapeId="0" xr:uid="{239EA25F-C042-224C-8583-7C08AAF67E1F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Eriogonum deflexum (obs 10/2, det 10/14 2026)</t>
+      </text>
+    </comment>
+    <comment ref="BG1" authorId="5" shapeId="0" xr:uid="{F5E67526-0680-034D-8892-EF4DAD13EEE1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    eriogonum abertianum</t>
+      </text>
+    </comment>
+    <comment ref="H7" authorId="6" shapeId="0" xr:uid="{841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -93,7 +111,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="97">
   <si>
     <t>plot</t>
   </si>
@@ -233,9 +251,6 @@
     <t>C23</t>
   </si>
   <si>
-    <t>ERIOGspp</t>
-  </si>
-  <si>
     <t>ENNDES</t>
   </si>
   <si>
@@ -336,19 +351,76 @@
   </si>
   <si>
     <t>C32</t>
+  </si>
+  <si>
+    <t>C47</t>
+  </si>
+  <si>
+    <t>BOUCUR</t>
+  </si>
+  <si>
+    <t>C37</t>
+  </si>
+  <si>
+    <t>C15</t>
+  </si>
+  <si>
+    <t>C41</t>
+  </si>
+  <si>
+    <t>ERIDEF</t>
+  </si>
+  <si>
+    <t>ERIABE</t>
+  </si>
+  <si>
+    <t>C30</t>
+  </si>
+  <si>
+    <t>C38</t>
+  </si>
+  <si>
+    <t>C29</t>
+  </si>
+  <si>
+    <t>C31</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>C9</t>
+  </si>
+  <si>
+    <t>C17</t>
+  </si>
+  <si>
+    <t>C35</t>
+  </si>
+  <si>
+    <t>C42</t>
+  </si>
+  <si>
+    <t>C19</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -732,6 +804,12 @@
   <threadedComment ref="AL1" dT="2026-09-07T18:56:57.85" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{9D1C2B35-25B3-DE40-B60B-62E13F57E42C}">
     <text>Atriplex elegans ("unk ama" on plot 98, by the road)</text>
   </threadedComment>
+  <threadedComment ref="AU1" dT="2026-10-14T21:24:44.18" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{239EA25F-C042-224C-8583-7C08AAF67E1F}">
+    <text>Eriogonum deflexum (obs 10/2, det 10/14 2026)</text>
+  </threadedComment>
+  <threadedComment ref="BG1" dT="2026-10-14T21:25:03.82" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{F5E67526-0680-034D-8892-EF4DAD13EEE1}">
+    <text>eriogonum abertianum</text>
+  </threadedComment>
   <threadedComment ref="H7" dT="2026-08-31T17:19:31.45" personId="{C061624E-6404-7544-875D-2039BE9EB8DC}" id="{841B92CE-65E8-0144-B0D7-EE8A5B2B0F57}">
     <text>incl. Hairy panic</text>
   </threadedComment>
@@ -740,10 +818,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD559584-3F3E-3149-A2F9-E170630AB5BF}">
-  <dimension ref="A1:BE75"/>
+  <dimension ref="A1:BG89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -883,40 +961,46 @@
         <v>43</v>
       </c>
       <c r="AU1" t="s">
+        <v>85</v>
+      </c>
+      <c r="AV1" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" t="s">
-        <v>47</v>
-      </c>
       <c r="AW1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="AX1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AY1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AZ1" t="s">
         <v>53</v>
       </c>
-      <c r="AZ1" t="s">
+      <c r="BA1" t="s">
         <v>54</v>
       </c>
-      <c r="BA1" t="s">
-        <v>55</v>
-      </c>
       <c r="BB1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="BC1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="BD1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="BE1" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="2" spans="1:57" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>81</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>97</v>
       </c>
@@ -985,7 +1069,7 @@
       <c r="AJ2" s="1"/>
       <c r="AK2" s="1"/>
     </row>
-    <row r="3" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>65</v>
       </c>
@@ -1054,7 +1138,7 @@
       <c r="AJ3" s="1"/>
       <c r="AK3" s="1"/>
     </row>
-    <row r="4" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>68</v>
       </c>
@@ -1123,7 +1207,7 @@
       <c r="AJ4" s="1"/>
       <c r="AK4" s="1"/>
     </row>
-    <row r="5" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>74</v>
       </c>
@@ -1192,7 +1276,7 @@
       <c r="AJ5" s="1"/>
       <c r="AK5" s="1"/>
     </row>
-    <row r="6" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>55</v>
       </c>
@@ -1247,7 +1331,7 @@
       <c r="AJ6" s="1"/>
       <c r="AK6" s="1"/>
     </row>
-    <row r="7" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>61</v>
       </c>
@@ -1304,7 +1388,7 @@
       <c r="AJ7" s="1"/>
       <c r="AK7" s="1"/>
     </row>
-    <row r="8" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>57</v>
       </c>
@@ -1363,7 +1447,7 @@
       <c r="AJ8" s="1"/>
       <c r="AK8" s="1"/>
     </row>
-    <row r="9" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>84</v>
       </c>
@@ -1412,7 +1496,7 @@
       <c r="AJ9" s="1"/>
       <c r="AK9" s="1"/>
     </row>
-    <row r="10" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>94</v>
       </c>
@@ -1465,7 +1549,7 @@
       <c r="AJ10" s="1"/>
       <c r="AK10" s="1"/>
     </row>
-    <row r="11" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>67</v>
       </c>
@@ -1514,7 +1598,7 @@
       <c r="AJ11" s="1"/>
       <c r="AK11" s="1"/>
     </row>
-    <row r="12" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>88</v>
       </c>
@@ -1561,7 +1645,7 @@
       <c r="AJ12" s="1"/>
       <c r="AK12" s="1"/>
     </row>
-    <row r="13" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>91</v>
       </c>
@@ -1616,7 +1700,7 @@
       <c r="AJ13" s="1"/>
       <c r="AK13" s="1"/>
     </row>
-    <row r="14" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>63</v>
       </c>
@@ -1669,7 +1753,7 @@
       <c r="AJ14" s="1"/>
       <c r="AK14" s="1"/>
     </row>
-    <row r="15" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>89</v>
       </c>
@@ -1718,7 +1802,7 @@
       <c r="AJ15" s="1"/>
       <c r="AK15" s="1"/>
     </row>
-    <row r="16" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:59" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>49</v>
       </c>
@@ -3753,7 +3837,7 @@
     </row>
     <row r="52" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="H52">
         <v>3</v>
@@ -3776,7 +3860,7 @@
     </row>
     <row r="53" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="I53">
         <v>20</v>
@@ -3790,7 +3874,7 @@
     </row>
     <row r="54" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C54">
         <v>10</v>
@@ -3828,7 +3912,7 @@
     </row>
     <row r="55" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="U55">
         <v>0.5</v>
@@ -3842,7 +3926,7 @@
     </row>
     <row r="56" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F56">
         <v>10</v>
@@ -3856,7 +3940,7 @@
     </row>
     <row r="57" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F57">
         <v>0.5</v>
@@ -3876,12 +3960,12 @@
     </row>
     <row r="58" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="59" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F59">
         <v>40</v>
@@ -3892,7 +3976,7 @@
     </row>
     <row r="60" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I60">
         <v>10</v>
@@ -3903,7 +3987,7 @@
     </row>
     <row r="61" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F61">
         <v>3</v>
@@ -3917,7 +4001,7 @@
     </row>
     <row r="62" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F62">
         <v>10</v>
@@ -3928,7 +4012,7 @@
     </row>
     <row r="63" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I63">
         <v>20</v>
@@ -3936,41 +4020,41 @@
     </row>
     <row r="64" spans="1:54" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
+        <v>65</v>
+      </c>
+      <c r="H64">
+        <v>0.5</v>
+      </c>
+      <c r="I64">
+        <v>3</v>
+      </c>
+      <c r="L64">
+        <v>10</v>
+      </c>
+      <c r="M64">
+        <v>0.5</v>
+      </c>
+      <c r="U64">
+        <v>3</v>
+      </c>
+      <c r="Y64">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="65" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A65" t="s">
         <v>66</v>
       </c>
-      <c r="H64">
-        <v>0.5</v>
-      </c>
-      <c r="I64">
-        <v>3</v>
-      </c>
-      <c r="L64">
-        <v>10</v>
-      </c>
-      <c r="M64">
-        <v>0.5</v>
-      </c>
-      <c r="U64">
-        <v>3</v>
-      </c>
-      <c r="Y64">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="65" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A65" t="s">
+      <c r="M65">
+        <v>10</v>
+      </c>
+      <c r="AZ65">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="66" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
         <v>67</v>
-      </c>
-      <c r="M65">
-        <v>10</v>
-      </c>
-      <c r="AZ65">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="66" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>68</v>
       </c>
       <c r="F66">
         <v>10</v>
@@ -3985,27 +4069,27 @@
         <v>3</v>
       </c>
     </row>
-    <row r="67" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
+        <v>68</v>
+      </c>
+      <c r="B67">
+        <v>0.5</v>
+      </c>
+      <c r="H67">
+        <v>0.5</v>
+      </c>
+      <c r="I67">
+        <v>3</v>
+      </c>
+      <c r="R67">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
         <v>69</v>
       </c>
-      <c r="B67">
-        <v>0.5</v>
-      </c>
-      <c r="H67">
-        <v>0.5</v>
-      </c>
-      <c r="I67">
-        <v>3</v>
-      </c>
-      <c r="R67">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="68" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>70</v>
-      </c>
       <c r="D68">
         <v>3</v>
       </c>
@@ -4025,46 +4109,46 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="69" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
+        <v>71</v>
+      </c>
+      <c r="F69">
+        <v>3</v>
+      </c>
+      <c r="I69">
+        <v>10</v>
+      </c>
+      <c r="K69">
+        <v>0.5</v>
+      </c>
+      <c r="AK69">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
         <v>72</v>
       </c>
-      <c r="F69">
-        <v>3</v>
-      </c>
-      <c r="I69">
-        <v>10</v>
-      </c>
-      <c r="K69">
-        <v>0.5</v>
-      </c>
-      <c r="AK69">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="70" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
+      <c r="M70">
+        <v>0.5</v>
+      </c>
+      <c r="S70">
+        <v>0.5</v>
+      </c>
+      <c r="U70">
+        <v>3</v>
+      </c>
+      <c r="AE70">
+        <v>3</v>
+      </c>
+      <c r="AU70">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
         <v>73</v>
-      </c>
-      <c r="M70">
-        <v>0.5</v>
-      </c>
-      <c r="S70">
-        <v>0.5</v>
-      </c>
-      <c r="U70">
-        <v>3</v>
-      </c>
-      <c r="AE70">
-        <v>3</v>
-      </c>
-      <c r="AU70">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="71" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>74</v>
       </c>
       <c r="I71">
         <v>20</v>
@@ -4073,30 +4157,30 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="72" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
+        <v>74</v>
+      </c>
+      <c r="I72">
+        <v>10</v>
+      </c>
+      <c r="O72">
+        <v>0.5</v>
+      </c>
+      <c r="U72">
+        <v>0.5</v>
+      </c>
+      <c r="AU72">
+        <v>0.5</v>
+      </c>
+      <c r="AX72">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
         <v>75</v>
       </c>
-      <c r="I72">
-        <v>10</v>
-      </c>
-      <c r="O72">
-        <v>0.5</v>
-      </c>
-      <c r="U72">
-        <v>0.5</v>
-      </c>
-      <c r="AU72">
-        <v>0.5</v>
-      </c>
-      <c r="AX72">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:57" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>76</v>
-      </c>
       <c r="G73">
         <v>0.5</v>
       </c>
@@ -4131,9 +4215,9 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="74" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F74">
         <v>0.5</v>
@@ -4157,11 +4241,264 @@
         <v>3</v>
       </c>
     </row>
-    <row r="75" spans="1:57" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:58" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
+        <v>79</v>
+      </c>
+      <c r="I75">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="76" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
         <v>80</v>
       </c>
-      <c r="I75">
+      <c r="F76">
+        <v>0.5</v>
+      </c>
+      <c r="H76">
+        <v>0.5</v>
+      </c>
+      <c r="I76">
+        <v>0.5</v>
+      </c>
+      <c r="K76">
+        <v>3</v>
+      </c>
+      <c r="M76">
+        <v>0.5</v>
+      </c>
+      <c r="O76">
+        <v>0.5</v>
+      </c>
+      <c r="Z76">
+        <v>3</v>
+      </c>
+      <c r="AH76">
+        <v>0.5</v>
+      </c>
+      <c r="AJ76">
+        <v>10</v>
+      </c>
+      <c r="AN76">
+        <v>0.5</v>
+      </c>
+      <c r="BF76">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="77" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>82</v>
+      </c>
+      <c r="H77">
+        <v>0.5</v>
+      </c>
+      <c r="I77">
+        <v>0.5</v>
+      </c>
+      <c r="J77">
+        <v>0.5</v>
+      </c>
+      <c r="T77">
+        <v>0.5</v>
+      </c>
+      <c r="AN77">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="78" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A78" t="s">
+        <v>83</v>
+      </c>
+      <c r="I78">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A79" t="s">
+        <v>84</v>
+      </c>
+      <c r="H79">
+        <v>0.5</v>
+      </c>
+      <c r="I79">
+        <v>10</v>
+      </c>
+      <c r="M79">
+        <v>0.5</v>
+      </c>
+      <c r="U79">
+        <v>10</v>
+      </c>
+      <c r="AK79">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="80" spans="1:58" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>87</v>
+      </c>
+      <c r="H80">
+        <v>0.5</v>
+      </c>
+      <c r="I80">
+        <v>40</v>
+      </c>
+      <c r="J80">
+        <v>0.5</v>
+      </c>
+      <c r="R80">
+        <v>0.5</v>
+      </c>
+      <c r="AC80">
+        <v>0.5</v>
+      </c>
+      <c r="AN80">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="81" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A81" t="s">
+        <v>88</v>
+      </c>
+      <c r="B81">
+        <v>20</v>
+      </c>
+      <c r="H81">
+        <v>10</v>
+      </c>
+      <c r="I81">
+        <v>10</v>
+      </c>
+      <c r="J81">
+        <v>0.5</v>
+      </c>
+      <c r="M81">
+        <v>3</v>
+      </c>
+      <c r="O81">
+        <v>3</v>
+      </c>
+      <c r="R81">
+        <v>0.5</v>
+      </c>
+      <c r="X81">
+        <v>3</v>
+      </c>
+      <c r="AN81">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="82" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>89</v>
+      </c>
+      <c r="I82">
+        <v>10</v>
+      </c>
+      <c r="AC82">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>90</v>
+      </c>
+      <c r="F83">
+        <v>3</v>
+      </c>
+      <c r="I83">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="84" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>91</v>
+      </c>
+      <c r="I84">
+        <v>50</v>
+      </c>
+      <c r="L84">
+        <v>0.5</v>
+      </c>
+      <c r="O84">
+        <v>3</v>
+      </c>
+      <c r="AE84">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="85" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>92</v>
+      </c>
+      <c r="H85">
+        <v>3</v>
+      </c>
+      <c r="Z85">
+        <v>0.5</v>
+      </c>
+      <c r="BB85">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>93</v>
+      </c>
+      <c r="F86">
+        <v>0.5</v>
+      </c>
+      <c r="K86">
+        <v>3</v>
+      </c>
+      <c r="M86">
+        <v>3</v>
+      </c>
+      <c r="AZ86">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>94</v>
+      </c>
+      <c r="B87">
+        <v>3</v>
+      </c>
+      <c r="H87">
+        <v>0.5</v>
+      </c>
+      <c r="I87">
+        <v>30</v>
+      </c>
+      <c r="J87">
+        <v>0.5</v>
+      </c>
+      <c r="Q87">
+        <v>0.5</v>
+      </c>
+      <c r="X87">
+        <v>0.5</v>
+      </c>
+      <c r="BC87">
+        <v>0.5</v>
+      </c>
+      <c r="BG87">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="89" spans="1:59" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>96</v>
+      </c>
+      <c r="AI89">
         <v>3</v>
       </c>
     </row>

</xml_diff>